<commit_message>
Intro to ML part 2
</commit_message>
<xml_diff>
--- a/wooclap/imports/optional/08_Intro_ML_Part_2_optional.xlsx
+++ b/wooclap/imports/optional/08_Intro_ML_Part_2_optional.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>L03-O03 · Deployment will predict future months for fields not used in training. The dataset has repeated monthly rows for each field. Which held-out evaluation matches both requirements?</t>
+          <t>L03-O03 · A yield model is trained on fields A–D using data from 2021–2023. We want to predict yields in 2024 for new fields. Which test set best checks this?</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -570,22 +570,22 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Randomly shuffle individual rows so the same fields and future dates can appear in training.</t>
+          <t>2024 records from fields A–D.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Train on earlier data from one group of fields, then evaluate later data from different fields.</t>
+          <t>2024 records from different fields, E–H.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Hold out later months but keep exactly the same fields in training and evaluation.</t>
+          <t>2021–2023 records from different fields, E–H.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Hold out field identities but allow later measurements to enter training before predicting earlier dates.</t>
+          <t>Unused 2021–2023 records from fields A–D, selected at random.</t>
         </is>
       </c>
       <c r="H3" s="3" t="n"/>

</xml_diff>